<commit_message>
sessao: 2026-05-07 — regen pos pipeline mestre (snapshot 69 devedores)
Snapshot apos `py -3.12 scripts\sincronizar_prodam.py`:
- 69 AUDITORIA_<DEVEDOR>.md + dashboard + resumo.json em AUDITORIA_COMPLETUDE/
- 69 dossies (md, html, xlsx, json, csv) em DOSSIES_MULTIFORMATO/

Numeros desta rodada:
- Score medio completude: 37,9%
- Total gaps documentais: 471
- Total divergencias: 17
- Alerta urgente: SES/SUSAM prescreve 2026-05-13 (6 dias) — R$ 14.748.048,96

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOSSIES_MULTIFORMATO/AMAZONPREV/dossie.xlsx
+++ b/DOSSIES_MULTIFORMATO/AMAZONPREV/dossie.xlsx
@@ -636,7 +636,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2020NE01268</t>
+          <t>2020NE01270</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>101856</v>
+        <v>680.3200000000001</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2020NE01270</t>
+          <t>2020NE01268</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>680.3200000000001</v>
+        <v>101856</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -804,12 +804,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024NE0001796</t>
+          <t>2024NE0001798</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -818,7 +818,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8269.24</v>
+        <v>17093.36</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -827,19 +827,19 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024NE0001797</t>
+          <t>2024NE0001799</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>106183.36</v>
+        <v>3645.46</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -857,19 +857,19 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024NE0001799</t>
+          <t>2024NE0001797</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3645.46</v>
+        <v>106183.36</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -887,19 +887,19 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024NE0001798</t>
+          <t>2024NE0001796</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>17093.36</v>
+        <v>8269.24</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -917,7 +917,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2017NE01015</t>
+          <t>2017NE01007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>10611.84</v>
+        <v>18986.95</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -969,14 +969,14 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00423, EM VIRTUDE DE SOBRA DE VALOR NÃO UTILIZADO.</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00059, EM VIRTUDE DE EXISTIR NOVO ADITIVO VIGENTE.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2017NE01014</t>
+          <t>2017NE01011</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>27828.43</v>
+        <v>9285.360000000001</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -995,14 +995,14 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00422, EM VIRTUDE DO VALOR NÃO TER SIDO UTILIZADO.</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00174, EM VIRTUDE DE EXISTIR NOVO ADITIVO VIGENTE.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2017NE01011</t>
+          <t>2017NE01014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>9285.360000000001</v>
+        <v>27828.43</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1021,14 +1021,14 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00174, EM VIRTUDE DE EXISTIR NOVO ADITIVO VIGENTE.</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00422, EM VIRTUDE DO VALOR NÃO TER SIDO UTILIZADO.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2017NE01007</t>
+          <t>2017NE01015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>18986.95</v>
+        <v>10611.84</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1047,17 +1047,21 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00059, EM VIRTUDE DE EXISTIR NOVO ADITIVO VIGENTE.</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00423, EM VIRTUDE DE SOBRA DE VALOR NÃO UTILIZADO.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2017NE00660</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>2017NE00661</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14/2014</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>29/08/2017</t>
@@ -1073,7 +1077,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO EMPENHO 2017NE00658 EM VIRTUDE DA VIGÊNCIA ESTÁ INCORRETA.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS.</t>
         </is>
       </c>
     </row>
@@ -1110,14 +1114,10 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2017NE00661</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>14/2014</t>
-        </is>
-      </c>
+          <t>2017NE00660</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>29/08/2017</t>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS.</t>
+          <t>ANULAÇÃO DO EMPENHO 2017NE00658 EM VIRTUDE DA VIGÊNCIA ESTÁ INCORRETA.</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1196,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025NE0001487</t>
+          <t>2025NE0001485</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1146.86</v>
+        <v>35636.68</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025NE0001485</t>
+          <t>2025NE0001487</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>35636.68</v>
+        <v>1146.86</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1279,14 +1279,14 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2022NE0001489</t>
+          <t>2022NE0001485</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1296,7 +1296,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>110826</v>
+        <v>1167.84</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1305,14 +1305,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DE SOBRA DA NOTA DE EMPENHO 2022NE0000083, VISTO QUE O VALOR NÃO SE CONSTITUIRÁ EM RESTOS A PAGAR, CONFORME DECRETO 46621 DE 11/11/22.</t>
+          <t>ANULAÇÃO DE SOBRA DA NOTA DE EMPENHO 2022NE0000076, VISTO QUE O VALOR NÃO SE CONSTITUIRÁ EM RESTOS A PAGAR, CONFORME DECRETO 46621 DE 11/11/22.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2022NE0001485</t>
+          <t>2022NE0001489</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1167.84</v>
+        <v>110826</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1331,14 +1331,14 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DE SOBRA DA NOTA DE EMPENHO 2022NE0000076, VISTO QUE O VALOR NÃO SE CONSTITUIRÁ EM RESTOS A PAGAR, CONFORME DECRETO 46621 DE 11/11/22.</t>
+          <t>ANULAÇÃO DE SOBRA DA NOTA DE EMPENHO 2022NE0000083, VISTO QUE O VALOR NÃO SE CONSTITUIRÁ EM RESTOS A PAGAR, CONFORME DECRETO 46621 DE 11/11/22.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2016NE00935</t>
+          <t>2016NE00923</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>10611.84</v>
+        <v>15461.47</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1364,7 +1364,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2016NE00933</t>
+          <t>2016NE00927</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>26204</v>
+        <v>171149.27</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2016NE00927</t>
+          <t>2016NE00933</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>171149.27</v>
+        <v>26204</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1416,7 +1416,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2016NE00923</t>
+          <t>2016NE00935</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>15461.47</v>
+        <v>10611.84</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1502,12 +1502,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2023NE0000371</t>
+          <t>2023NE0000379</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1516,7 +1516,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>16404.57</v>
+        <v>424733.44</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1525,19 +1525,19 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 2</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 417/2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2023NE0000379</t>
+          <t>2023NE0000371</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1546,7 +1546,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>424733.44</v>
+        <v>16404.57</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 417/2</t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 2</t>
         </is>
       </c>
     </row>
@@ -1622,12 +1622,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2024NE0001889</t>
+          <t>2024NE0001886</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4134.62</v>
+        <v>17818.34</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1645,19 +1645,19 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2024NE0001887</t>
+          <t>2024NE0001888</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>53091.68</v>
+        <v>1822.73</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1675,19 +1675,19 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2024NE0001888</t>
+          <t>2024NE0001887</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1822.73</v>
+        <v>53091.68</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1705,19 +1705,19 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2024NE0001886</t>
+          <t>2024NE0001889</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>17818.34</v>
+        <v>4134.62</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1735,19 +1735,19 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2021NE0001029</t>
+          <t>2021NE0001030</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>18/2018</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>42411.9</v>
+        <v>1167.84</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1765,19 +1765,19 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO</t>
+          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E P</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2021NE0001030</t>
+          <t>2021NE0001029</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>18/2018</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1167.84</v>
+        <v>42411.9</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1795,7 +1795,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E P</t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO</t>
         </is>
       </c>
     </row>
@@ -1862,12 +1862,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2017NE00421</t>
+          <t>2017NE00422</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>P.53/2017</t>
+          <t>11/2014</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>23808.72</v>
+        <v>27828.43</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO DE SISTEMAS WEBSERVICES PARA A AMAZONPREV EM 2017.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
         </is>
       </c>
     </row>
@@ -1922,12 +1922,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2017NE00422</t>
+          <t>2017NE00421</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>11/2014</t>
+          <t>P.53/2017</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>27828.43</v>
+        <v>23808.72</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO DE SISTEMAS WEBSERVICES PARA A AMAZONPREV EM 2017.</t>
         </is>
       </c>
     </row>
@@ -2102,12 +2102,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2024NE0001021</t>
+          <t>2024NE0001022</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3645.46</v>
+        <v>34186.72</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
@@ -2162,12 +2162,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2024NE0001022</t>
+          <t>2024NE0001021</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>34186.72</v>
+        <v>3645.46</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
@@ -2312,10 +2312,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2021NE0000112</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
+          <t>2021NE0000111</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>1/2020</t>
+        </is>
+      </c>
       <c r="C60" t="inlineStr">
         <is>
           <t>15/02/2021</t>
@@ -2331,21 +2335,17 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO EMPENHO 2021NE00023, EM VIRTUDE DO ADITIVO DE PRAZO PARA CONCLUSÃO DAS ATIVIDADES DE 2020. O VALOR VAI COMPOR O ADITIVO, VISTO QUE NÃO SERÁ UTILIZADO MAIS NO CONTRATO VIGENTE.</t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE DIGITALIZAÇÃO DE DOCUMENTOS, COM FORNECIMENTO DE EQUIPAMENTOS, ARMAZENAMENTOS EM STORAGE E SOFTWARE, DE ACORDO COM EDITAL, TERMO DE REFERÊNCIA, PROJETO BÁSICO E PROPOSTA TÉCNI</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2021NE0000111</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>1/2020</t>
-        </is>
-      </c>
+          <t>2021NE0000112</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>15/02/2021</t>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE DIGITALIZAÇÃO DE DOCUMENTOS, COM FORNECIMENTO DE EQUIPAMENTOS, ARMAZENAMENTOS EM STORAGE E SOFTWARE, DE ACORDO COM EDITAL, TERMO DE REFERÊNCIA, PROJETO BÁSICO E PROPOSTA TÉCNI</t>
+          <t>ANULAÇÃO DO EMPENHO 2021NE00023, EM VIRTUDE DO ADITIVO DE PRAZO PARA CONCLUSÃO DAS ATIVIDADES DE 2020. O VALOR VAI COMPOR O ADITIVO, VISTO QUE NÃO SERÁ UTILIZADO MAIS NO CONTRATO VIGENTE.</t>
         </is>
       </c>
     </row>
@@ -2428,12 +2428,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2025NE0000818</t>
+          <t>2025NE0000816</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2442,7 +2442,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>8269.24</v>
+        <v>111237.68</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2451,19 +2451,19 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2025NE0000815</t>
+          <t>2025NE0000817</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>35636.68</v>
+        <v>3823</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2481,19 +2481,19 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2025NE0000817</t>
+          <t>2025NE0000815</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2502,7 +2502,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>3823</v>
+        <v>35636.68</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2511,19 +2511,19 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2025NE0000816</t>
+          <t>2025NE0000818</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>111237.68</v>
+        <v>8269.24</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2541,14 +2541,14 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2015NE00053</t>
+          <t>2015NE00065</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2571,14 +2571,14 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO REFERIDO EMPENHO EM VIRTUDE DA MODALIDADE DE EMPENHO ESTÁ INCORRETA.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO REGIME PRÓPRIO DE PREVIDÊN</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2015NE00065</t>
+          <t>2015NE00053</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2601,28 +2601,24 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO REGIME PRÓPRIO DE PREVIDÊN</t>
+          <t>ANULAÇÃO DO REFERIDO EMPENHO EM VIRTUDE DA MODALIDADE DE EMPENHO ESTÁ INCORRETA.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2021NE0001187</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1/2020</t>
-        </is>
-      </c>
+          <t>2021NE0001188</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>13/12/2021</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>971615.23</v>
+        <v>334829.73</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2631,24 +2627,28 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE DIGITALIZAÇÃO DE DOCUMENTOS, COM FORNECIMENTO DE EQUIPAMENTOS, ARMAZENAMENTOS EM STORAGE E SOFTWARE, DE ACORDO COM EDITAL, TERMO DE REFERÊNCIA, PROJETO BÁSICO E PROPOSTA TÉCNI</t>
+          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE MATCHER DE IMAGENS DE IMPRESSÕES FACIAIS EM FORMATO WEB SERVICE PARA SER CONSUMIDO PELO SISTEMA DE PROVA DE VIDA DE ATIVOS, APOSENTADOS E PENSIONIST</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2021NE0001188</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
+          <t>2021NE0001187</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>1/2020</t>
+        </is>
+      </c>
       <c r="C71" t="inlineStr">
         <is>
           <t>13/12/2021</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>334829.73</v>
+        <v>971615.23</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2657,28 +2657,24 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE MATCHER DE IMAGENS DE IMPRESSÕES FACIAIS EM FORMATO WEB SERVICE PARA SER CONSUMIDO PELO SISTEMA DE PROVA DE VIDA DE ATIVOS, APOSENTADOS E PENSIONIST</t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE DIGITALIZAÇÃO DE DOCUMENTOS, COM FORNECIMENTO DE EQUIPAMENTOS, ARMAZENAMENTOS EM STORAGE E SOFTWARE, DE ACORDO COM EDITAL, TERMO DE REFERÊNCIA, PROJETO BÁSICO E PROPOSTA TÉCNI</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2019NE00922</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>8/2019</t>
-        </is>
-      </c>
+          <t>2019NE00920</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>13/08/2019</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>17301.45</v>
+        <v>12169.61</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2687,24 +2683,28 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE REFORMULAÇÃO DO WEBSITE DA FUNDAÇÃO AMAZONPREV, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PO</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2019NE00917 PARA CORREÇÃO DE VALORES E DO OBJETO DA CONTRATAÇÃO.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2019NE00920</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
+          <t>2019NE00922</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>8/2019</t>
+        </is>
+      </c>
       <c r="C73" t="inlineStr">
         <is>
           <t>13/08/2019</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>12169.61</v>
+        <v>17301.45</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2019NE00917 PARA CORREÇÃO DE VALORES E DO OBJETO DA CONTRATAÇÃO.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE REFORMULAÇÃO DO WEBSITE DA FUNDAÇÃO AMAZONPREV, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PO</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2750,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2025NE0002276</t>
+          <t>2025NE0002277</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2764,7 +2764,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>111237.68</v>
+        <v>8709.200000000001</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2773,19 +2773,19 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV. TC: 0003/2024 AD: 01.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2025NE0002277</t>
+          <t>2025NE0002276</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>8709.200000000001</v>
+        <v>111237.68</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2803,19 +2803,19 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV. TC: 0003/2024 AD: 01.</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2025NE0000410</t>
+          <t>2025NE0000411</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2824,7 +2824,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>111237.68</v>
+        <v>3823</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2833,19 +2833,19 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2025NE0000409</t>
+          <t>2025NE0000412</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2854,7 +2854,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35636.68</v>
+        <v>8269.24</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2863,19 +2863,19 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2025NE0000412</t>
+          <t>2025NE0000409</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2884,7 +2884,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>8269.24</v>
+        <v>35636.68</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2893,19 +2893,19 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2025NE0000411</t>
+          <t>2025NE0000410</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2914,7 +2914,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3823</v>
+        <v>111237.68</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2923,19 +2923,19 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2024NE0001428</t>
+          <t>2024NE0001427</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2944,7 +2944,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1822.73</v>
+        <v>17093.36</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2953,19 +2953,19 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2024NE0001426</t>
+          <t>2024NE0001425</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>53091.68</v>
+        <v>4134.62</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2983,19 +2983,19 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2024NE0001425</t>
+          <t>2024NE0001426</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3004,7 +3004,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>4134.62</v>
+        <v>53091.68</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -3013,19 +3013,19 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2024NE0001427</t>
+          <t>2024NE0001428</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3034,7 +3034,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17093.36</v>
+        <v>1822.73</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
@@ -3136,12 +3136,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025NE0001948</t>
+          <t>2025NE0001950</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>17818.34</v>
+        <v>4354.6</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV. TC: 0003/2024 AD: 01.</t>
         </is>
       </c>
     </row>
@@ -3196,12 +3196,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2025NE0001950</t>
+          <t>2025NE0001948</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3210,7 +3210,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>4354.6</v>
+        <v>17818.34</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -3219,19 +3219,19 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV. TC: 0003/2024 AD: 01.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025NE0001741</t>
+          <t>2025NE0001739</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3240,7 +3240,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>4354.6</v>
+        <v>17818.34</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -3249,7 +3249,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV. TC: 0003/2024 AD: 01.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
@@ -3286,12 +3286,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2025NE0001739</t>
+          <t>2025NE0001741</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3300,7 +3300,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>17818.34</v>
+        <v>4354.6</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV. TC: 0003/2024 AD: 01.</t>
         </is>
       </c>
     </row>
@@ -3462,12 +3462,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2015NE00015</t>
+          <t>2015NE00018</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>11/2014</t>
+          <t>14/2014</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3476,7 +3476,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>23733.7</v>
+        <v>985383.12</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3522,12 +3522,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2015NE00018</t>
+          <t>2015NE00015</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>14/2014</t>
+          <t>11/2014</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3536,7 +3536,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>985383.12</v>
+        <v>23733.7</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -3582,10 +3582,14 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2018NE00302</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr"/>
+          <t>2018NE00288</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2/2018</t>
+        </is>
+      </c>
       <c r="C103" t="inlineStr">
         <is>
           <t>04/04/2018</t>
@@ -3601,7 +3605,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2018NE00288, EM VIRTUDE DA DATA DA VIGÊNCIA DO CONTRATO ESTAR INCORRETA.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
         </is>
       </c>
     </row>
@@ -3638,14 +3642,10 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2018NE00288</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>2/2018</t>
-        </is>
-      </c>
+          <t>2018NE00302</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
           <t>04/04/2018</t>
@@ -3661,19 +3661,19 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2018NE00288, EM VIRTUDE DA DATA DA VIGÊNCIA DO CONTRATO ESTAR INCORRETA.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2024NE0000339</t>
+          <t>2024NE0000337</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3682,7 +3682,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>106183.36</v>
+        <v>3645.46</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
@@ -3728,12 +3728,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2024NE0000337</t>
+          <t>2024NE0000339</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3742,7 +3742,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>3645.46</v>
+        <v>106183.36</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
@@ -3784,12 +3784,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2021NE0000017</t>
+          <t>2021NE0000032</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2/2018</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3798,7 +3798,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>106248</v>
+        <v>211402.8</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3807,19 +3807,19 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2021NE0000023</t>
+          <t>2021NE0000029</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>1/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3828,7 +3828,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>322258.41</v>
+        <v>20409.48</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3837,19 +3837,19 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DIGITALIZAÇÃO DE DOCUMENTOS, COM FORNECIMENTO DE EQUIPAMENTOS, ARMAZENAMENTOS EM STORAGE E SOFTWARE, DE ACORDO COM EDITAL, TERMO DE REF</t>
+          <t>CONTRATAÇÃO DA PRODAM P/PPRESTAÇÃO DE SERVIÇOS LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET), C</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2021NE0000025</t>
+          <t>2021NE0000056</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10/2019</t>
+          <t>18/2018</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3858,7 +3858,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1526090.72</v>
+        <v>59667.63</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3867,19 +3867,19 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM O PROJE</t>
+          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E P</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2021NE0000056</t>
+          <t>2021NE0000025</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>18/2018</t>
+          <t>10/2019</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3888,7 +3888,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>59667.63</v>
+        <v>1526090.72</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3897,19 +3897,19 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E P</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM O PROJE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2021NE0000029</t>
+          <t>2021NE0000023</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>1/2020</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3918,7 +3918,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>20409.48</v>
+        <v>322258.41</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3927,19 +3927,19 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DA PRODAM P/PPRESTAÇÃO DE SERVIÇOS LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET), C</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DIGITALIZAÇÃO DE DOCUMENTOS, COM FORNECIMENTO DE EQUIPAMENTOS, ARMAZENAMENTOS EM STORAGE E SOFTWARE, DE ACORDO COM EDITAL, TERMO DE REF</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2021NE0000032</t>
+          <t>2021NE0000017</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>2/2018</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>211402.8</v>
+        <v>106248</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3957,19 +3957,19 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2016NE00066</t>
+          <t>2016NE00058</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>14/2014</t>
+          <t>13/2014</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3978,7 +3978,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>985383.12</v>
+        <v>36390</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3987,7 +3987,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM O PROJET</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO À INTERNET, COM VELOCIDADE DE 5 MBPS, CONFORME PROJETO BÁSICO E PROPOSTA TÉCNICA E DE PREÇOS.</t>
         </is>
       </c>
     </row>
@@ -4024,12 +4024,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2016NE00058</t>
+          <t>2016NE00066</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>13/2014</t>
+          <t>14/2014</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -4038,7 +4038,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>36390</v>
+        <v>985383.12</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -4047,19 +4047,19 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO À INTERNET, COM VELOCIDADE DE 5 MBPS, CONFORME PROJETO BÁSICO E PROPOSTA TÉCNICA E DE PREÇOS.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM O PROJET</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2024NE0000646</t>
+          <t>2024NE0000647</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>1/2023</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4068,7 +4068,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>34186.72</v>
+        <v>106183.36</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
         </is>
       </c>
     </row>
@@ -4114,12 +4114,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2024NE0000647</t>
+          <t>2024NE0000646</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>1/2023</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -4128,7 +4128,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>106183.36</v>
+        <v>34186.72</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -4137,7 +4137,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>PREST. SERV. EXECUÇÃO DE SIST. INF, CAD E FOLHA DE PAGTO DE PESSOAL DOS SERV ATIVOS DA AMAZONPREV, INCLUINDO SERV SUP TÉC EM SIST DE INF CONF. ESP CONST NO PB, PP E PORTARIA. PARECER JURÍDICO N° 4491/</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
@@ -4260,12 +4260,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2014NE00513</t>
+          <t>2014NE00556</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>5/2011</t>
+          <t>11/2014</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>290338.86</v>
+        <v>33227.18</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -4283,19 +4283,19 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Contrato No. 5/2011 - RPPS - Regime Próprio de Previdência Social</t>
+          <t>Contrato No. 11/2014</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2014NE00556</t>
+          <t>2014NE00513</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11/2014</t>
+          <t>5/2011</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -4304,7 +4304,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>33227.18</v>
+        <v>290338.86</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4313,28 +4313,24 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Contrato No. 11/2014</t>
+          <t>Contrato No. 5/2011 - RPPS - Regime Próprio de Previdência Social</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2017NE00174</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>3/2016</t>
-        </is>
-      </c>
+          <t>2017NE00173</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
           <t>02/03/2017</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>79588.8</v>
+        <v>59691.6</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -4343,24 +4339,28 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO À INTERNET, COM VELOCIDADE DE 30 MBPS</t>
+          <t>ANULAÇÃO DO EMPENHO 2017NE00005 PARA UTILIZAÇÃO DO RECURSO NO ADITIVO A SER REALIZADO COM A PRODAM PARA AUMENTO DA FRANQUIA DE 20MBPS PARA 30 MBPS SEM ÕNUS ADICIONAL PARA A CONTRATANTE.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2017NE00173</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr"/>
+          <t>2017NE00174</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>3/2016</t>
+        </is>
+      </c>
       <c r="C129" t="inlineStr">
         <is>
           <t>02/03/2017</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>59691.6</v>
+        <v>79588.8</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4369,19 +4369,19 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO EMPENHO 2017NE00005 PARA UTILIZAÇÃO DO RECURSO NO ADITIVO A SER REALIZADO COM A PRODAM PARA AUMENTO DA FRANQUIA DE 20MBPS PARA 30 MBPS SEM ÕNUS ADICIONAL PARA A CONTRATANTE.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO À INTERNET, COM VELOCIDADE DE 30 MBPS</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2025NE0000020</t>
+          <t>2025NE0000023</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>3/2024</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -4390,7 +4390,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>35636.68</v>
+        <v>8269.24</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -4399,14 +4399,14 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2025NE0000022</t>
+          <t>2025NE0000024</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>1093.61</v>
+        <v>2676.14</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -4429,14 +4429,14 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2025NE0000024</t>
+          <t>2025NE0000022</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -4450,7 +4450,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>2676.14</v>
+        <v>1093.61</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4459,19 +4459,19 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET). TC: 0013/2020 AD: 04.</t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2025NE0000023</t>
+          <t>2025NE0000020</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>3/2024</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -4480,7 +4480,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>8269.24</v>
+        <v>35636.68</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4489,19 +4489,19 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA PRESTAR OS SERVIÇOS DE LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A UTILIZAÇÃO DO GESTOR DE CONTEÚDO WEB – GERWEB, PARA A FUNDAÇÃO AMAZONPREV.</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2024NE0000027</t>
+          <t>2024NE0000010</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>2551.85</v>
+        <v>34186.72</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -4519,24 +4519,28 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
+          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2024NE0000043</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr"/>
+          <t>2024NE0000009</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>13/2020</t>
+        </is>
+      </c>
       <c r="C135" t="inlineStr">
         <is>
           <t>02/01/2024</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>2551.85</v>
+        <v>668.34</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -4545,7 +4549,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Anulação de Saldo para correção da Data de Emissão da Nota de Empenho.</t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 2</t>
         </is>
       </c>
     </row>
@@ -4582,21 +4586,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2024NE0000009</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>13/2020</t>
-        </is>
-      </c>
+          <t>2024NE0000043</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
           <t>02/01/2024</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>668.34</v>
+        <v>2551.85</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4605,19 +4605,19 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 2</t>
+          <t>Anulação de Saldo para correção da Data de Emissão da Nota de Empenho.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2024NE0000010</t>
+          <t>2024NE0000027</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>34186.72</v>
+        <v>2551.85</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -4635,19 +4635,19 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DA PRODAM PARA PREST DE SERV DE ACESSO A INTERNET, CONF. ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO. PARECER JURÍDICO N° </t>
+          <t>CONT. PRODAM P/ PREST. DE SERV. LICENÇA DE USO DE SIST DE INF, COMP A DISP. GESTOR DE CONT. WEB P/ PUB DE INF INTERNAS (INTRANET), CONF. ESPECIFICAÇÕES CONSTANTES DO PB, PT E PP. PARECER JURÍDICO N° 4</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2023NE0000015</t>
+          <t>2023NE0000043</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>12/2020</t>
+          <t>13/2020</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -4656,7 +4656,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>68179.23</v>
+        <v>4799.85</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -4665,19 +4665,19 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO.</t>
+          <t>PRESTAÇÃO DE SERVIÇOS LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET), CONFORME ESPECIFICAÇÕES CO</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2023NE0000043</t>
+          <t>2023NE0000015</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>13/2020</t>
+          <t>12/2020</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -4686,7 +4686,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>4799.85</v>
+        <v>68179.23</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -4695,19 +4695,19 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>PRESTAÇÃO DE SERVIÇOS LICENÇA DE USO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A DISPONIBILIZAÇÃO DE GESTOR DE CONTEÚDO WEB PARA PUBLICAÇÃO DE INFORMAÇÕES INTERNAS (INTRANET), CONFORME ESPECIFICAÇÕES CO</t>
+          <t>CONTRATAÇÃO DA PRODAM PARA PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE DISPENSA DE LICITAÇÃO.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2020NE00027</t>
+          <t>2020NE00028</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>8/2019</t>
+          <t>18/2018</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -4716,7 +4716,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>11905.53</v>
+        <v>59667.63</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -4725,19 +4725,19 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE REFORMULAÇÃO DO WEBSITE DA FUNDAÇÃO AMAZONPREV, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PO</t>
+          <t xml:space="preserve">CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E </t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2020NE00024</t>
+          <t>2020NE00025</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>2/2018</t>
+          <t>10/2019</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4746,7 +4746,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>101856</v>
+        <v>1526090.72</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM O PROJE</t>
         </is>
       </c>
     </row>
@@ -4792,12 +4792,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2020NE00025</t>
+          <t>2020NE00024</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>10/2019</t>
+          <t>2/2018</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -4806,7 +4806,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>1526090.72</v>
+        <v>101856</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4815,19 +4815,19 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM O PROJE</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2020NE00028</t>
+          <t>2020NE00027</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>18/2018</t>
+          <t>8/2019</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -4836,7 +4836,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>59667.63</v>
+        <v>11905.53</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -4845,19 +4845,19 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E </t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE REFORMULAÇÃO DO WEBSITE DA FUNDAÇÃO AMAZONPREV, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PO</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2019NE00009</t>
+          <t>2019NE00063</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>14/2014</t>
+          <t>18/2018</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -4866,7 +4866,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>1002036.08</v>
+        <v>57708.95</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4875,19 +4875,19 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, CONFORME PROJETO BÁS</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME AS ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2019NE00003</t>
+          <t>2019NE00002</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>13/2014</t>
+          <t>2/2018</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -4896,7 +4896,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>99486</v>
+        <v>98154</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4905,19 +4905,19 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, COM VELOCIDADE DE 30MBPS, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTA</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2019NE00002</t>
+          <t>2019NE00003</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2/2018</t>
+          <t>13/2014</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4926,7 +4926,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>98154</v>
+        <v>99486</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4935,19 +4935,19 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DESENVOLVIMENTO EVOLUTIVO DE SISTEMAS DE INFORMAÇÃO, COMPREENDENDO A ANÁLISE E DESENVOLVIMENTO DE FUNCIONALIDADES E RELATÓRIOS NOS SIST</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, COM VELOCIDADE DE 30MBPS, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTA</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2019NE00063</t>
+          <t>2019NE00009</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>18/2018</t>
+          <t>14/2014</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4956,7 +4956,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>57708.95</v>
+        <v>1002036.08</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4965,19 +4965,19 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE PROTOCOLO EM PLATAFORMA WEB (SPROWEB), CONFORME AS ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOLHA DE PAGAMENTO E ROTINAS DO RPPS, CONFORME PROJETO BÁS</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2018NE00032</t>
+          <t>2018NE00034</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11/2014</t>
+          <t>3/2016</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -4986,7 +4986,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>19877.45</v>
+        <v>99486</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4995,7 +4995,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇO DE ACESSO A INTERNET COM VELOCIDADE DE 30 MBPS</t>
         </is>
       </c>
     </row>
@@ -5032,12 +5032,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2018NE00034</t>
+          <t>2018NE00032</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>3/2016</t>
+          <t>11/2014</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -5046,7 +5046,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>99486</v>
+        <v>19877.45</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -5055,28 +5055,24 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇO DE ACESSO A INTERNET COM VELOCIDADE DE 30 MBPS</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2017NE00059</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>11/2014</t>
-        </is>
-      </c>
+          <t>2017NE00048</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
       <c r="C153" t="inlineStr">
         <is>
           <t>02/01/2017</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>18986.95</v>
+        <v>985383.12</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5085,28 +5081,24 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00019, EM VIRTUDE DE INFORMAÇÕES INCONSISTENTES PRESENTES NO REFERIDO EMPENHO.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2017NE00064</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>14/2014</t>
-        </is>
-      </c>
+          <t>2017NE00043</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
       <c r="C154" t="inlineStr">
         <is>
           <t>02/01/2017</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>985383.12</v>
+        <v>18986.95</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -5115,19 +5107,19 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, GESTÃO E PROCESSAMENTO DE FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM PROJETO BÁSICO E PROPO</t>
+          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00012, EM VIRTUDE DE INFORMAÇÕES INCONSISTENTES PRESENTES NO REFERIDO EMPENHO.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2017NE00005</t>
+          <t>2017NE00012</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>3/2016</t>
+          <t>11/2014</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -5136,7 +5128,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>99486</v>
+        <v>18986.95</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -5145,7 +5137,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO À INTERNET, COM VELOCIDADE DE 20 MBPS, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORT</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
         </is>
       </c>
     </row>
@@ -5182,12 +5174,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2017NE00012</t>
+          <t>2017NE00005</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>11/2014</t>
+          <t>3/2016</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -5196,7 +5188,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>18986.95</v>
+        <v>99486</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -5205,24 +5197,28 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO À INTERNET, COM VELOCIDADE DE 20 MBPS, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORT</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2017NE00043</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr"/>
+          <t>2017NE00064</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>14/2014</t>
+        </is>
+      </c>
       <c r="C158" t="inlineStr">
         <is>
           <t>02/01/2017</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>18986.95</v>
+        <v>985383.12</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -5231,24 +5227,28 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00012, EM VIRTUDE DE INFORMAÇÕES INCONSISTENTES PRESENTES NO REFERIDO EMPENHO.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DE SISTEMA DE INFORMAÇÃO, GESTÃO E PROCESSAMENTO DE FOLHA DE PAGAMENTO E ROTINAS DO RPPS, DE ACORDO COM PROJETO BÁSICO E PROPO</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2017NE00048</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr"/>
+          <t>2017NE00059</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>11/2014</t>
+        </is>
+      </c>
       <c r="C159" t="inlineStr">
         <is>
           <t>02/01/2017</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>985383.12</v>
+        <v>18986.95</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -5257,19 +5257,19 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DA NOTA DE EMPENHO 2017NE00019, EM VIRTUDE DE INFORMAÇÕES INCONSISTENTES PRESENTES NO REFERIDO EMPENHO.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE INFORMÁTICA DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E PREÇOS E PORTARIA DE DISPENSA D</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2014NE00003</t>
+          <t>2014NE00004</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>7/2009</t>
+          <t>8/2010</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -5278,7 +5278,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>23733.7</v>
+        <v>67172.16</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -5287,7 +5287,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Contrato N. 007/2009 - Serviços Eventuais de Informatica</t>
+          <t>Contrato No. 8/2010 - Acesso Computador / Internet 4 Mbps - MetroMAO</t>
         </is>
       </c>
     </row>
@@ -5324,12 +5324,12 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2014NE00004</t>
+          <t>2014NE00003</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>8/2010</t>
+          <t>7/2009</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -5338,7 +5338,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>67172.16</v>
+        <v>23733.7</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -5347,7 +5347,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Contrato No. 8/2010 - Acesso Computador / Internet 4 Mbps - MetroMAO</t>
+          <t>Contrato N. 007/2009 - Serviços Eventuais de Informatica</t>
         </is>
       </c>
     </row>
@@ -5564,17 +5564,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2018NE00175</t>
-        </is>
-      </c>
-      <c r="B170" t="inlineStr"/>
+          <t>2018NE00182</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>11/2014</t>
+        </is>
+      </c>
       <c r="C170" t="inlineStr">
         <is>
           <t>01/03/2018</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>815399.4399999999</v>
+        <v>19877.45</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -5583,19 +5587,19 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO EMPENHO 2018NE00033 PARA MUDANÇA DO ELEMENTO DE DESPESA, CONFORME ORIENTAÇÃO TÉCNICA N° 12/18 GINS/SEFAZ.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE ADJUDICAÇÃO.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2018NE00184</t>
+          <t>2018NE00183</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>3/2016</t>
+          <t>14/2014</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -5604,7 +5608,7 @@
         </is>
       </c>
       <c r="D171" t="n">
-        <v>59691.6</v>
+        <v>815399.4399999999</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -5613,14 +5617,14 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, COM VELOCIDADE DE 30 MBPS, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E E PREÇOS E PORTA</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DO SISTEMA DE INFORMAÇÃO, COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOPAG E ROTINAS DO RPPS, CONFORME PB E PT.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2018NE00176</t>
+          <t>2018NE00174</t>
         </is>
       </c>
       <c r="B172" t="inlineStr"/>
@@ -5630,7 +5634,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>59691.6</v>
+        <v>19877.45</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -5639,14 +5643,14 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO EMPENHO 2018NE00034 PARA MUDANÇA DO ELEMENTO DE DESPESA, CONFORME ORIENTAÇÃO TÉCNICA N° 12/18 GINS/SEFAZ.</t>
+          <t>ANULAÇÃO DO EMPENHO 2018NE00032 PARA MUDANÇA DO ELEMENTO DE DESPESA, CONFORME ORIENTAÇÃO TÉCNICA N° 12/18 GINS/SEFAZ.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2018NE00174</t>
+          <t>2018NE00176</t>
         </is>
       </c>
       <c r="B173" t="inlineStr"/>
@@ -5656,7 +5660,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>19877.45</v>
+        <v>59691.6</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -5665,19 +5669,19 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>ANULAÇÃO DO EMPENHO 2018NE00032 PARA MUDANÇA DO ELEMENTO DE DESPESA, CONFORME ORIENTAÇÃO TÉCNICA N° 12/18 GINS/SEFAZ.</t>
+          <t>ANULAÇÃO DO EMPENHO 2018NE00034 PARA MUDANÇA DO ELEMENTO DE DESPESA, CONFORME ORIENTAÇÃO TÉCNICA N° 12/18 GINS/SEFAZ.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2018NE00183</t>
+          <t>2018NE00184</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>14/2014</t>
+          <t>3/2016</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -5686,7 +5690,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>815399.4399999999</v>
+        <v>59691.6</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -5695,28 +5699,24 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE EXECUÇÃO DO SISTEMA DE INFORMAÇÃO, COMPREENDENDO A GESTÃO E PROCESSAMENTO DA FOPAG E ROTINAS DO RPPS, CONFORME PB E PT.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE ACESSO A INTERNET, COM VELOCIDADE DE 30 MBPS, CONFORME ESPECIFICAÇÕES CONSTANTES DO PROJETO BÁSICO, PROPOSTA TÉCNICA E E PREÇOS E PORTA</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2018NE00182</t>
-        </is>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>11/2014</t>
-        </is>
-      </c>
+          <t>2018NE00175</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr"/>
       <c r="C175" t="inlineStr">
         <is>
           <t>01/03/2018</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>19877.45</v>
+        <v>815399.4399999999</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5725,7 +5725,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE FORMA EVENTUAL, CONFORME ESPECIFICAÇÕES CONSTANTES NO PROJETO BÁSICO, PROPOSTA TÉCNICA E DE PREÇOS E PORTARIA DE ADJUDICAÇÃO.</t>
+          <t>ANULAÇÃO DO EMPENHO 2018NE00033 PARA MUDANÇA DO ELEMENTO DE DESPESA, CONFORME ORIENTAÇÃO TÉCNICA N° 12/18 GINS/SEFAZ.</t>
         </is>
       </c>
     </row>

</xml_diff>